<commit_message>
Allow student-chosen Year and Section with 3-column admin creation
</commit_message>
<xml_diff>
--- a/frontend/public/sample_student_bulk_import.xlsx
+++ b/frontend/public/sample_student_bulk_import.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E6"/>
+  <dimension ref="A1:C11"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -409,12 +409,6 @@
       <c r="C1" t="str">
         <v>DOB</v>
       </c>
-      <c r="D1" t="str">
-        <v>Year</v>
-      </c>
-      <c r="E1" t="str">
-        <v>Section</v>
-      </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
@@ -426,12 +420,6 @@
       <c r="C2" t="str">
         <v>2005-02-14</v>
       </c>
-      <c r="D2">
-        <v>2</v>
-      </c>
-      <c r="E2" t="str">
-        <v>A</v>
-      </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
@@ -443,12 +431,6 @@
       <c r="C3" t="str">
         <v>2005-07-28</v>
       </c>
-      <c r="D3">
-        <v>2</v>
-      </c>
-      <c r="E3" t="str">
-        <v>A</v>
-      </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
@@ -460,12 +442,6 @@
       <c r="C4" t="str">
         <v>2005-10-12</v>
       </c>
-      <c r="D4">
-        <v>2</v>
-      </c>
-      <c r="E4" t="str">
-        <v>B</v>
-      </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
@@ -477,12 +453,6 @@
       <c r="C5" t="str">
         <v>2005-04-03</v>
       </c>
-      <c r="D5">
-        <v>2</v>
-      </c>
-      <c r="E5" t="str">
-        <v>B</v>
-      </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
@@ -494,16 +464,65 @@
       <c r="C6" t="str">
         <v>2006-01-20</v>
       </c>
-      <c r="D6">
-        <v>1</v>
-      </c>
-      <c r="E6" t="str">
-        <v>A</v>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>71762405032</v>
+      </c>
+      <c r="B7" t="str">
+        <v>MANIKANDAN P</v>
+      </c>
+      <c r="C7" t="str">
+        <v>2006-08-16</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>71762405033</v>
+      </c>
+      <c r="B8" t="str">
+        <v>NITHISH KUMAR T</v>
+      </c>
+      <c r="C8" t="str">
+        <v>2006-11-09</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>71762405034</v>
+      </c>
+      <c r="B9" t="str">
+        <v>POOJA S</v>
+      </c>
+      <c r="C9" t="str">
+        <v>2006-05-24</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>71762205051</v>
+      </c>
+      <c r="B10" t="str">
+        <v>SANTHOSH C</v>
+      </c>
+      <c r="C10" t="str">
+        <v>2004-09-19</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>71762205052</v>
+      </c>
+      <c r="B11" t="str">
+        <v>YUVASRI N</v>
+      </c>
+      <c r="C11" t="str">
+        <v>2004-12-08</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E6"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C11"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat(auth): transition student onboarding to whitelist-only import and self-signup with live verification
</commit_message>
<xml_diff>
--- a/frontend/public/sample_student_bulk_import.xlsx
+++ b/frontend/public/sample_student_bulk_import.xlsx
@@ -3,7 +3,8 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
-    <sheet name="Students" sheetId="1" r:id="rId1"/>
+    <sheet name="Eligible Students" sheetId="1" r:id="rId1"/>
+    <sheet name="Instructions" sheetId="2" r:id="rId2"/>
   </sheets>
 </workbook>
 </file>
@@ -32,8 +33,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:vt="http://schemas.openxmlformats.org/officeDocument/2006/docPropsVTypes">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="56" formatCode="&quot;上午/下午 &quot;hh&quot;時&quot;mm&quot;分&quot;ss&quot;秒 &quot;"/>
+    <numFmt numFmtId="60" formatCode="dd-mm-yyyy"/>
   </numFmts>
   <fonts count="1">
     <font>
@@ -64,8 +66,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="60" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -397,16 +400,17 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C11"/>
+  <dimension ref="A1:B6"/>
+  <cols>
+    <col min="1" max="1" width="20.83203125" customWidth="1"/>
+    <col min="2" max="2" width="15.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
         <v>Register Number</v>
       </c>
       <c r="B1" t="str">
-        <v>Name</v>
-      </c>
-      <c r="C1" t="str">
         <v>DOB</v>
       </c>
     </row>
@@ -414,115 +418,115 @@
       <c r="A2" t="str">
         <v>71762305041</v>
       </c>
-      <c r="B2" t="str">
-        <v>ANITHA R</v>
-      </c>
-      <c r="C2" t="str">
-        <v>2005-02-14</v>
+      <c r="B2" s="1">
+        <v>38397</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
         <v>71762305042</v>
       </c>
-      <c r="B3" t="str">
-        <v>BHARATHI K</v>
-      </c>
-      <c r="C3" t="str">
-        <v>2005-07-28</v>
+      <c r="B3" s="1">
+        <v>38547</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
         <v>71762305043</v>
       </c>
-      <c r="B4" t="str">
-        <v>DINESH S</v>
-      </c>
-      <c r="C4" t="str">
-        <v>2005-10-12</v>
+      <c r="B4" s="1">
+        <v>38637</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
         <v>71762305044</v>
       </c>
-      <c r="B5" t="str">
-        <v>GOKUL PRASATH V</v>
-      </c>
-      <c r="C5" t="str">
-        <v>2005-04-03</v>
+      <c r="B5" s="1">
+        <v>38316</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>71762405031</v>
+        <v>71762305045</v>
+      </c>
+      <c r="B6" s="1">
+        <v>38598</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:B6"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:B8"/>
+  <cols>
+    <col min="1" max="1" width="25.83203125" customWidth="1"/>
+    <col min="2" max="2" width="70.83203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>AI&amp;DS Portal - Student Whitelist Ingestion Instructions</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>Required Columns:</v>
+      </c>
+      <c r="B3" t="str">
+        <v>2 Columns Only (Register Number, DOB)</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>1. Register Number:</v>
+      </c>
+      <c r="B4" t="str">
+        <v>Must be formatted as Text (no scientific notation, e.g. 71762305041)</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>2. DOB:</v>
+      </c>
+      <c r="B5" t="str">
+        <v>Valid calendar birth date (DD-MM-YYYY, YYYY-MM-DD, or Excel Date cell)</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>Age limit:</v>
       </c>
       <c r="B6" t="str">
-        <v>KAVITHA M</v>
-      </c>
-      <c r="C6" t="str">
-        <v>2006-01-20</v>
+        <v>Student must be between 15 and 40 years old</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>71762405032</v>
-      </c>
-      <c r="B7" t="str">
-        <v>MANIKANDAN P</v>
-      </c>
-      <c r="C7" t="str">
-        <v>2006-08-16</v>
+        <v/>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>71762405033</v>
+        <v>Note:</v>
       </c>
       <c r="B8" t="str">
-        <v>NITHISH KUMAR T</v>
-      </c>
-      <c r="C8" t="str">
-        <v>2006-11-09</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="str">
-        <v>71762405034</v>
-      </c>
-      <c r="B9" t="str">
-        <v>POOJA S</v>
-      </c>
-      <c r="C9" t="str">
-        <v>2006-05-24</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="str">
-        <v>71762205051</v>
-      </c>
-      <c r="B10" t="str">
-        <v>SANTHOSH C</v>
-      </c>
-      <c r="C10" t="str">
-        <v>2004-09-19</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="str">
-        <v>71762205052</v>
-      </c>
-      <c r="B11" t="str">
-        <v>YUVASRI N</v>
-      </c>
-      <c r="C11" t="str">
-        <v>2004-12-08</v>
+        <v>Do NOT add Name, Year, Section, or Email columns. Students will self-register their account details.</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C11"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:B8"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
fix(security): resolve open audit issues (U1-U3, O1-O8, M3-M8, X1-X8)
</commit_message>
<xml_diff>
--- a/frontend/public/sample_student_bulk_import.xlsx
+++ b/frontend/public/sample_student_bulk_import.xlsx
@@ -3,8 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
-    <sheet name="Eligible Students" sheetId="1" r:id="rId1"/>
-    <sheet name="Instructions" sheetId="2" r:id="rId2"/>
+    <sheet name="Students" sheetId="1" r:id="rId1"/>
   </sheets>
 </workbook>
 </file>
@@ -33,9 +32,8 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:vt="http://schemas.openxmlformats.org/officeDocument/2006/docPropsVTypes">
-  <numFmts count="2">
+  <numFmts count="1">
     <numFmt numFmtId="56" formatCode="&quot;上午/下午 &quot;hh&quot;時&quot;mm&quot;分&quot;ss&quot;秒 &quot;"/>
-    <numFmt numFmtId="60" formatCode="dd-mm-yyyy"/>
   </numFmts>
   <fonts count="1">
     <font>
@@ -66,9 +64,8 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="60" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -401,10 +398,6 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:B6"/>
-  <cols>
-    <col min="1" max="1" width="20.83203125" customWidth="1"/>
-    <col min="2" max="2" width="15.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -416,42 +409,42 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>71762305041</v>
-      </c>
-      <c r="B2" s="1">
-        <v>38397</v>
+        <v>SAMPLE00001</v>
+      </c>
+      <c r="B2" t="str">
+        <v>01-01-2005</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>71762305042</v>
-      </c>
-      <c r="B3" s="1">
-        <v>38547</v>
+        <v>SAMPLE00002</v>
+      </c>
+      <c r="B3" t="str">
+        <v>02-02-2005</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>71762305043</v>
-      </c>
-      <c r="B4" s="1">
-        <v>38637</v>
+        <v>SAMPLE00003</v>
+      </c>
+      <c r="B4" t="str">
+        <v>03-03-2005</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>71762305044</v>
-      </c>
-      <c r="B5" s="1">
-        <v>38316</v>
+        <v>SAMPLE00004</v>
+      </c>
+      <c r="B5" t="str">
+        <v>04-04-2005</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>71762305045</v>
-      </c>
-      <c r="B6" s="1">
-        <v>38598</v>
+        <v>SAMPLE00005</v>
+      </c>
+      <c r="B6" t="str">
+        <v>05-05-2005</v>
       </c>
     </row>
   </sheetData>
@@ -459,74 +452,4 @@
     <ignoredError numberStoredAsText="1" sqref="A1:B6"/>
   </ignoredErrors>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B8"/>
-  <cols>
-    <col min="1" max="1" width="25.83203125" customWidth="1"/>
-    <col min="2" max="2" width="70.83203125" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="str">
-        <v>AI&amp;DS Portal - Student Whitelist Ingestion Instructions</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="str">
-        <v>Required Columns:</v>
-      </c>
-      <c r="B3" t="str">
-        <v>2 Columns Only (Register Number, DOB)</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="str">
-        <v>1. Register Number:</v>
-      </c>
-      <c r="B4" t="str">
-        <v>Must be formatted as Text (no scientific notation, e.g. 71762305041)</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="str">
-        <v>2. DOB:</v>
-      </c>
-      <c r="B5" t="str">
-        <v>Valid calendar birth date (DD-MM-YYYY, YYYY-MM-DD, or Excel Date cell)</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="str">
-        <v>Age limit:</v>
-      </c>
-      <c r="B6" t="str">
-        <v>Student must be between 15 and 40 years old</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="str">
-        <v>Note:</v>
-      </c>
-      <c r="B8" t="str">
-        <v>Do NOT add Name, Year, Section, or Email columns. Students will self-register their account details.</v>
-      </c>
-    </row>
-  </sheetData>
-  <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B8"/>
-  </ignoredErrors>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
feat: update support email to aiandds.support@gmail.com and enforce DD/MM/YYYY date format across all DOB fields
</commit_message>
<xml_diff>
--- a/frontend/public/sample_student_bulk_import.xlsx
+++ b/frontend/public/sample_student_bulk_import.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
-    <sheet name="Students" sheetId="1" r:id="rId1"/>
+    <sheet name="Eligible_Students" sheetId="1" r:id="rId1"/>
   </sheets>
 </workbook>
 </file>
@@ -412,7 +412,7 @@
         <v>SAMPLE00001</v>
       </c>
       <c r="B2" t="str">
-        <v>01-01-2005</v>
+        <v>01/01/2005</v>
       </c>
     </row>
     <row r="3">
@@ -420,7 +420,7 @@
         <v>SAMPLE00002</v>
       </c>
       <c r="B3" t="str">
-        <v>02-02-2005</v>
+        <v>02/02/2005</v>
       </c>
     </row>
     <row r="4">
@@ -428,7 +428,7 @@
         <v>SAMPLE00003</v>
       </c>
       <c r="B4" t="str">
-        <v>03-03-2005</v>
+        <v>03/03/2005</v>
       </c>
     </row>
     <row r="5">
@@ -436,7 +436,7 @@
         <v>SAMPLE00004</v>
       </c>
       <c r="B5" t="str">
-        <v>04-04-2005</v>
+        <v>04/04/2005</v>
       </c>
     </row>
     <row r="6">
@@ -444,7 +444,7 @@
         <v>SAMPLE00005</v>
       </c>
       <c r="B6" t="str">
-        <v>05-05-2005</v>
+        <v>05/05/2005</v>
       </c>
     </row>
   </sheetData>

</xml_diff>